<commit_message>
Fictional German demo receipts, English Excel output, invoices paid up to 14 days later
- Demo receipts and bank CSV use invented shops only, each stamped MUSTER
- Added donation confirmation, household-service invoice and pharmacy receipt
- Excel sheets and labels in English (German tax terms kept in brackets)
- Matching accepts a bank line 3 days before to 14 days after the receipt date
- README demo results updated (9 receipts, 8 read correctly, café misread caught)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/DEMO_Belegbuch_2026Q3.xlsx
+++ b/samples/DEMO_Belegbuch_2026Q3.xlsx
@@ -7,9 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Belege" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Fehlende Belege" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Schaetzung" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Receipts" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Missing receipts" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Estimate" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,88 +425,88 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="9" customWidth="1" min="5" max="5"/>
-    <col width="23" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="35" customWidth="1" min="8" max="8"/>
-    <col width="34" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="21" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="8" max="8"/>
+    <col width="44" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="15" customWidth="1" min="12" max="12"/>
     <col width="50" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Datum</t>
+          <t>Date</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Händler</t>
+          <t>Shop</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Betrag</t>
+          <t>Total €</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>MwSt 19%</t>
+          <t>VAT 19%</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>MwSt 7%</t>
+          <t>VAT 7%</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Kategorie (Vorschlag)</t>
+          <t>Category (suggested)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Zahlung</t>
+          <t>Paid by</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Positionen</t>
+          <t>Items</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Datei</t>
+          <t>File</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Gelesen als</t>
+          <t>Read as</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Bankbuchung</t>
+          <t>Bank line</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>≈ Steuerersparnis €</t>
+          <t>≈ tax saved €</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>Bitte prüfen</t>
+          <t>Please check</t>
         </is>
       </c>
     </row>
@@ -518,7 +518,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Deutsche Bahn</t>
+          <t>Regio-Bahn Muster</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -529,7 +529,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Fahrtkosten</t>
+          <t>Fahrtkosten (commuting)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -544,7 +544,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>db_deutschlandticket_2026-07.pdf</t>
+          <t>regio-bahn_deutschlandticket_2026-07.pdf</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -570,7 +570,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>THALIA Buchhandlung</t>
+          <t>Buchhandlung Lesezeichen</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -581,12 +581,12 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Fachliteratur</t>
+          <t>Fachliteratur (professional books)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>card</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -596,7 +596,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>thalia_2026-07-08.jpg</t>
+          <t>lesezeichen_2026-07-08.jpg</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -622,7 +622,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Amazon EU S.a r.l.</t>
+          <t>Versandhaus Muster GmbH</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -633,7 +633,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Arbeitsmittel</t>
+          <t>Arbeitsmittel (work equipment)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -648,7 +648,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>amazon_rechnung_2026-07-11.pdf</t>
+          <t>versandhaus-muster_rechnung_2026-07-11.pdf</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -669,130 +669,120 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Udemy</t>
+          <t>Aktion Musterhilfe e.V.</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>19.99</v>
-      </c>
-      <c r="D5" t="n">
-        <v>3.19</v>
+        <v>50</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Fortbildung</t>
+          <t>Spende (donation)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>card</t>
+          <t>transfer</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Python for Data Analysis (course)</t>
+          <t>Geldzuwendung</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>udemy_2026-08-14.eml</t>
+          <t>musterhilfe_spende_2026-07-20.pdf</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>email text</t>
+          <t>pdf text</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
-        </is>
-      </c>
-      <c r="L5" t="n">
-        <v>0</v>
-      </c>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-03</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Cafe Muster</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="n">
-        <v>17.84</v>
-      </c>
-      <c r="D6" s="2" t="n">
-        <v>3.34</v>
-      </c>
-      <c r="E6" s="2" t="n"/>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>Privat</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>Cappuccino, Croissant, BAR</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>cafe_2026-09-03.jpg</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Muster Haushaltsservice</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>120</v>
+      </c>
+      <c r="D6" t="n">
+        <v>19.16</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Haushaltsnahe Dienstleistung (household service)</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>transfer</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Fensterreinigung Wohnung Musterstr. 3</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>haushaltsservice_rechnung_2026-08.jpg</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
         <is>
           <t>photo</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>nicht gefunden</t>
-        </is>
-      </c>
-      <c r="L6" s="2" t="inlineStr"/>
-      <c r="M6" s="2" t="inlineStr">
-        <is>
-          <t>VAT larger than possible for this total; VAT 3.34 does not fit 19% of 17.84 (expected 2.85)</t>
-        </is>
-      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>MediaMarkt Frankfurt</t>
+          <t>Lernplattform Muster</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>79</v>
+        <v>19.99</v>
       </c>
       <c r="D7" t="n">
-        <v>12.61</v>
+        <v>3.19</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Arbeitsmittel</t>
+          <t>Fortbildung (training)</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -802,28 +792,185 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>USB Headset Pro</t>
+          <t>Online-Kurs: Python fuer Datenanalyse</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>mediamarkt_2026-09-11.jpg</t>
+          <t>lernplattform_2026-08-14.eml</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>photo</t>
+          <t>email text</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="L7" t="n">
         <v>0</v>
       </c>
       <c r="M7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Apotheke am Markt</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>27.8</v>
+      </c>
+      <c r="D8" t="n">
+        <v>4.44</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Krankheitskosten (medical)</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>card</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Ibuprofen 400 20st, Nasenspray, Vitamin D3 Tropfen</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>apotheke-am-markt_2026-08-22.jpg</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>photo</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Cafe Muster</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>13.34</v>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>1.34</v>
+      </c>
+      <c r="E9" s="2" t="n"/>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Privat (private)</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Cappuccino, Croissant, BAR</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>cafe-muster_2026-09-03.jpg</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>photo</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>not found</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr"/>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>VAT 1.34 does not fit 19% of 13.34 (expected 2.13)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Elektro Funke</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>79</v>
+      </c>
+      <c r="D10" t="n">
+        <v>12.61</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Arbeitsmittel (work equipment)</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>card</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>USB Headset Pro</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>elektro-funke_2026-09-11.jpg</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>photo</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="L10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -836,82 +983,82 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="36" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="31" customWidth="1" min="2" max="2"/>
+    <col width="29" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Datum</t>
+          <t>Date</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Empfänger</t>
+          <t>Payee</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Verwendungszweck</t>
+          <t>Purpose</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Betrag</t>
+          <t>Amount €</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Wahrscheinlich steuerlich relevant</t>
+          <t>Probably tax-relevant</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Aktion Musterhilfe e.V.</t>
+          <t>Regio-Bahn Muster GmbH</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Spende</t>
+          <t>Deutschlandticket August</t>
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>-50</v>
+        <v>-63</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Spende</t>
+          <t>Fahrtkosten (commuting)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>DB Vertrieb GmbH</t>
+          <t>Regio-Bahn Muster GmbH</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Deutschlandticket August</t>
+          <t>Deutschlandticket September</t>
         </is>
       </c>
       <c r="D3" s="2" t="n">
@@ -919,256 +1066,181 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Fahrtkosten</t>
+          <t>Fahrtkosten (commuting)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Muster Haushaltsservice</t>
+          <t>Gewerkschaft Muster</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Rechnung 2026-081 Fensterreinigung</t>
+          <t>Mitgliedsbeitrag Q3</t>
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>-120</v>
+        <v>-45</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Haushaltsnahe Dienstleistung</t>
+          <t>Gewerkschaft (union fee)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-22</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Apotheke am Markt</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Kartenzahlung Apotheke</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="n">
-        <v>-27.8</v>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Krankheitskosten</t>
-        </is>
-      </c>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Wohnbau Muster GmbH</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Miete Juli 2026</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>-950</v>
+      </c>
+      <c r="E5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-02</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>DB Vertrieb GmbH</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Deutschlandticket September</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="n">
-        <v>-63</v>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Fahrtkosten</t>
-        </is>
-      </c>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Frischmarkt Muster</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Kartenzahlung Frischmarkt</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>-42.37</v>
+      </c>
+      <c r="E6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Gewerkschaft Muster</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Mitgliedsbeitrag Q3</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="n">
-        <v>-45</v>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>Gewerkschaft</t>
-        </is>
-      </c>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Wohnbau Muster GmbH</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Miete August 2026</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>-950</v>
+      </c>
+      <c r="E7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Wohnbau Muster GmbH</t>
+          <t>Netz Muster Telekommunikation</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Miete Juli 2026</t>
+          <t>Internet August</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>-950</v>
+        <v>-39.95</v>
       </c>
       <c r="E8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>REWE Markt</t>
+          <t>Wohnbau Muster GmbH</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Kartenzahlung REWE</t>
+          <t>Miete September 2026</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>-42.37</v>
+        <v>-950</v>
       </c>
       <c r="E9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Wohnbau Muster GmbH</t>
+          <t>Netz Muster Telekommunikation</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Miete August 2026</t>
+          <t>Internet September</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>-950</v>
+        <v>-39.95</v>
       </c>
       <c r="E10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Telekom Deutschland</t>
+          <t>Lieferservice Muster</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Internet August</t>
+          <t>Kartenzahlung Essen</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>-39.95</v>
+        <v>-23.5</v>
       </c>
       <c r="E11" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Wohnbau Muster GmbH</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Miete September 2026</t>
-        </is>
-      </c>
-      <c r="D12" t="n">
-        <v>-950</v>
-      </c>
-      <c r="E12" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>2026-09-06</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Telekom Deutschland</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Internet September</t>
-        </is>
-      </c>
-      <c r="D13" t="n">
-        <v>-39.95</v>
-      </c>
-      <c r="E13" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Lieferando</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Kartenzahlung Essen</t>
-        </is>
-      </c>
-      <c r="D14" t="n">
-        <v>-23.5</v>
-      </c>
-      <c r="E14" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1184,20 +1256,20 @@
   <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="58" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Grobe Schätzung — keine Steuerberatung. Der Steuerberater entscheidet.</t>
+          <t>Rough estimate, not tax advice. Your Steuerberater decides.</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Werbungskosten aus Belegen</t>
+          <t>Work expenses from receipts (Werbungskosten) €</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -1207,7 +1279,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Arbeitnehmer-Pauschbetrag (§9a EStG)</t>
+          <t>Employee lump sum (Arbeitnehmer-Pauschbetrag, §9a EStG) €</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -1217,7 +1289,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Noch bis zum Pauschbetrag (erst danach sparen Belege Steuer)</t>
+          <t>Still to go before receipts save any tax €</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -1227,7 +1299,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>zu versteuerndes Einkommen (Eingabe, z. B. letzter Steuerbescheid)</t>
+          <t>Taxable income (input, e.g. last Steuerbescheid) €</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -1237,7 +1309,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Je 100 € Werbungskosten über dem Pauschbetrag ≈ € Steuer weniger</t>
+          <t>Each €100 of work expenses above the lump sum ≈ € less tax</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -1247,7 +1319,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>≈ Steuerersparnis durch diese Belege (§32a EStG 2026)</t>
+          <t>≈ Tax saved by these receipts (§32a EStG 2026) €</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -1257,7 +1329,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Nicht berücksichtigt: Solidaritätszuschlag, Kirchensteuer, Zusammenveranlagung, Sonderausgaben, §35a, Höchstbeträge. Nur Belege der Kategorien Arbeitsmittel, Fachliteratur, Fahrtkosten, Fortbildung, Gewerkschaft.</t>
+          <t>Not included: solidarity surcharge, church tax, joint assessment, special expenses, §35a, caps. Only receipts in: Arbeitsmittel (work equipment), Fachliteratur (professional books), Fahrtkosten (commuting), Fortbildung (training), Gewerkschaft (union fee).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Spending sheet: Gemma 4 labels and summarizes, code computes and checks every number
- src/spending.py: bank lines labelled in one local Gemma call (cached), totals,
  shares, months and recurring payments by code, summary written from those
  numbers only, and a check that flags any number the code did not compute
- Fake ING quarter grows to 48 lines; README and screenshots updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/DEMO_Belegbuch_2026Q3.xlsx
+++ b/samples/DEMO_Belegbuch_2026Q3.xlsx
@@ -10,6 +10,7 @@
     <sheet name="Receipts" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Missing receipts" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Estimate" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Spending" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -56,10 +57,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -983,7 +987,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1119,128 +1123,695 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Frischmarkt Muster</t>
+          <t>Fitness Muster</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Kartenzahlung Frischmarkt</t>
+          <t>Mitgliedschaft Juli</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>-42.37</v>
+        <v>-29.9</v>
       </c>
       <c r="E6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Wohnbau Muster GmbH</t>
+          <t>Streamdienst Muster</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Miete August 2026</t>
+          <t>Abo Standard</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>-950</v>
+        <v>-13.99</v>
       </c>
       <c r="E7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Netz Muster Telekommunikation</t>
+          <t>Frischmarkt Muster</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Internet August</t>
+          <t>Kartenzahlung Frischmarkt</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>-39.95</v>
+        <v>-42.37</v>
       </c>
       <c r="E8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Wohnbau Muster GmbH</t>
+          <t>Netz Muster Telekommunikation</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Miete September 2026</t>
+          <t>Internet Juli</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>-950</v>
+        <v>-39.95</v>
       </c>
       <c r="E9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Netz Muster Telekommunikation</t>
+          <t>Biomarkt Muster</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Internet September</t>
+          <t>Kartenzahlung Biomarkt</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>-39.95</v>
+        <v>-31.2</v>
       </c>
       <c r="E10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Trattoria Muster</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Kartenzahlung Restaurant</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>-38.5</v>
+      </c>
+      <c r="E11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Frischmarkt Muster</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Kartenzahlung Frischmarkt</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>-56.8</v>
+      </c>
+      <c r="E12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Lieferservice Muster</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Kartenzahlung Essen</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>-21.9</v>
+      </c>
+      <c r="E13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Frischmarkt Muster</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Kartenzahlung Frischmarkt</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>-47.15</v>
+      </c>
+      <c r="E14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Drogerie Muster</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Kartenzahlung Drogerie</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>-18.45</v>
+      </c>
+      <c r="E15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Kino Muster</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Kartenzahlung Kino</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>-24</v>
+      </c>
+      <c r="E16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Wohnbau Muster GmbH</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Miete August 2026</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>-950</v>
+      </c>
+      <c r="E17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Frischmarkt Muster</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Kartenzahlung Frischmarkt</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>-61.04</v>
+      </c>
+      <c r="E18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Fitness Muster</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Mitgliedschaft August</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>-29.9</v>
+      </c>
+      <c r="E19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Streamdienst Muster</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Abo Standard</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>-13.99</v>
+      </c>
+      <c r="E20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Netz Muster Telekommunikation</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Internet August</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>-39.95</v>
+      </c>
+      <c r="E21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Biomarkt Muster</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Kartenzahlung Biomarkt</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>-27.6</v>
+      </c>
+      <c r="E22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Frischmarkt Muster</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Kartenzahlung Frischmarkt</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>-52.33</v>
+      </c>
+      <c r="E23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Modehaus Muster</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Kartenzahlung Bekleidung</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>-79.95</v>
+      </c>
+      <c r="E24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Trattoria Muster</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Kartenzahlung Restaurant</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>-44.2</v>
+      </c>
+      <c r="E25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Lieferservice Muster</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Kartenzahlung Essen</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>-26.4</v>
+      </c>
+      <c r="E26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Frischmarkt Muster</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Kartenzahlung Frischmarkt</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>-39.98</v>
+      </c>
+      <c r="E27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Wohnbau Muster GmbH</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Miete September 2026</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>-950</v>
+      </c>
+      <c r="E28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Fitness Muster</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Mitgliedschaft September</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>-29.9</v>
+      </c>
+      <c r="E29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Streamdienst Muster</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Abo Standard</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>-13.99</v>
+      </c>
+      <c r="E30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Frischmarkt Muster</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Kartenzahlung Frischmarkt</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>-58.12</v>
+      </c>
+      <c r="E31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Netz Muster Telekommunikation</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Internet September</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>-39.95</v>
+      </c>
+      <c r="E32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Biomarkt Muster</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Kartenzahlung Biomarkt</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>-33.75</v>
+      </c>
+      <c r="E33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Cafe Muster</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Kartenzahlung Cafe</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>-11.8</v>
+      </c>
+      <c r="E34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Frischmarkt Muster</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Kartenzahlung Frischmarkt</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>-49.61</v>
+      </c>
+      <c r="E35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Drogerie Muster</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Kartenzahlung Drogerie</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>-22.1</v>
+      </c>
+      <c r="E36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B37" t="inlineStr">
         <is>
           <t>Lieferservice Muster</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C37" t="inlineStr">
         <is>
           <t>Kartenzahlung Essen</t>
         </is>
       </c>
-      <c r="D11" t="n">
+      <c r="D37" t="n">
         <v>-23.5</v>
       </c>
-      <c r="E11" t="inlineStr"/>
+      <c r="E37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Trattoria Muster</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Kartenzahlung Restaurant</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>-52</v>
+      </c>
+      <c r="E38" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1336,4 +1907,363 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C34"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="90" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Summary by Gemma 4 (local). Every number below the summary was computed by code.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="110" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>The total income for the quarter was €8,550.00, with total spending amounting to €4,734.95. This means that spending accounted for 55.4% of the income, leaving a remainder of €3,815.05. The largest expense category was Rent at €2,850.00, which represents 60.2% of total spending. Spending was distributed across three months: €1,667.10, €1,596.13, and €1,471.72.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Check: every number in the summary matches the code's numbers</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Income €</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>8550</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Spending €</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>4734.95</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Left over €</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>3815.05</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Spending as % of income</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>55.4</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="inlineStr">
+        <is>
+          <t>Total €</t>
+        </is>
+      </c>
+      <c r="C10" s="1" t="inlineStr">
+        <is>
+          <t>Share of spending %</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Rent</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>2850</v>
+      </c>
+      <c r="C11" t="n">
+        <v>60.2</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Groceries</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>499.95</v>
+      </c>
+      <c r="C12" t="n">
+        <v>10.6</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Shopping</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>389.4</v>
+      </c>
+      <c r="C13" t="n">
+        <v>8.199999999999999</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Eating out</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>218.3</v>
+      </c>
+      <c r="C14" t="n">
+        <v>4.6</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>189</v>
+      </c>
+      <c r="C15" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Leisure</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>155.67</v>
+      </c>
+      <c r="C16" t="n">
+        <v>3.3</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Household services</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>120</v>
+      </c>
+      <c r="C17" t="n">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Phone &amp; internet</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>119.85</v>
+      </c>
+      <c r="C18" t="n">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>69.98</v>
+      </c>
+      <c r="C19" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Donations</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>50</v>
+      </c>
+      <c r="C20" t="n">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>45</v>
+      </c>
+      <c r="C21" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>27.8</v>
+      </c>
+      <c r="C22" t="n">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t>Month</t>
+        </is>
+      </c>
+      <c r="B24" s="1" t="inlineStr">
+        <is>
+          <t>Spending €</t>
+        </is>
+      </c>
+      <c r="C24" s="1" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>1667.1</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>1596.13</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>1471.72</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="1" t="inlineStr">
+        <is>
+          <t>Every month (recurring)</t>
+        </is>
+      </c>
+      <c r="B29" s="1" t="inlineStr">
+        <is>
+          <t>Amount €</t>
+        </is>
+      </c>
+      <c r="C29" s="1" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Wohnbau Muster GmbH</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>950</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Regio-Bahn Muster GmbH</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Netz Muster Telekommunikation</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>39.95</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Fitness Muster</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>29.9</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Streamdienst Muster</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>13.99</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>